<commit_message>
Update gq-spinoff - Planejamento e Controle do Projeto.xlsx
Atualização - Planejamento e Controle do Projeto
</commit_message>
<xml_diff>
--- a/gq-spinoff/6.Gerenciamento de Projeto/gq-spinoff - Planejamento e Controle do Projeto.xlsx
+++ b/gq-spinoff/6.Gerenciamento de Projeto/gq-spinoff - Planejamento e Controle do Projeto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Amanda\EstudosDev\htmlCss\GQ-SPINOFF\gq-spinoff\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD75A14-BE56-439F-8D9D-1A179E61A464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0B8695-D5E5-4BF1-BB95-B5978C4E219B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="2" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -4738,7 +4738,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="253">
   <si>
     <t>Equipe</t>
   </si>
@@ -5513,12 +5513,6 @@
     <t>O prazo de conclusão entre foi definido para antes da data de entrega oficial</t>
   </si>
   <si>
-    <t>Diagrama de arquitetura</t>
-  </si>
-  <si>
-    <t>UC01 - Gerenciar checklist de verificação</t>
-  </si>
-  <si>
     <t>Especificar, Analisar e Projetar UC01-Gerenciar checklist de verificação (escolhido para testar a arquitetura)</t>
   </si>
   <si>
@@ -5540,31 +5534,58 @@
     <t>Modelar o UC01-Gerenciar checklist de verificação</t>
   </si>
   <si>
-    <t>Modelar, Implementare Testar o UC01-Gerenciar checklist de verificação</t>
-  </si>
-  <si>
     <t>Modelar UC02-Verificar projeto</t>
   </si>
   <si>
-    <t>Modelar, Implementart e Testar o UC02-Verificar projeto</t>
-  </si>
-  <si>
     <t>Modelar UC03-Criar verificação</t>
   </si>
   <si>
-    <t>Modelar, Implementart e Testar o UC03-Criar verificação</t>
-  </si>
-  <si>
     <t>Modelar UC04-Visualizar indicador de aderência ao process</t>
   </si>
   <si>
-    <t>Modelar, Implementart e Testar o UC04-Visualizar indicador de aderência ao process</t>
-  </si>
-  <si>
     <t>Modelar UC05-Consultar resultados por fases</t>
   </si>
   <si>
-    <t>Modelar, Implementart e Testar o UC05-Consultar resultados por fases</t>
+    <t>Diagrama de arquitetura, diagrama de classes, histórias de usuário</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC01-Gerenciar checklist de verificação</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC02-Verificar projeto</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC03-Criar verificação</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC04-Visualizar indicador de aderência ao process</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC05-Consultar resultados por fases</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC02-Verificar projeto e UC03-Criar verificação</t>
+  </si>
+  <si>
+    <t>Modelar, Implementar e Testar o UC04-Visualizar indicador de aderência ao processo e UC05-Consultar resultados por fases</t>
+  </si>
+  <si>
+    <t>Preparar e executar testes, corrigir defeitos</t>
+  </si>
+  <si>
+    <t>Planejar implantação e criar material de suporte e treinamento</t>
+  </si>
+  <si>
+    <t>Em execução</t>
+  </si>
+  <si>
+    <t>Estudar novas tecnologias</t>
+  </si>
+  <si>
+    <t>Dividir as tarefas de acordo com a tecnologia que será utilizada</t>
+  </si>
+  <si>
+    <t>1. Dividir as novas tecnologias que cada um irá aprender 2. Separar as atividades de acordo com a familiriadade com a tecnologia que será utilizada</t>
   </si>
 </sst>
 </file>
@@ -5583,7 +5604,7 @@
     <numFmt numFmtId="172" formatCode="#,##0.00&quot; &quot;;&quot;-&quot;#,##0.00&quot; &quot;;&quot; -&quot;#&quot; &quot;;@&quot; &quot;"/>
     <numFmt numFmtId="173" formatCode="[$R$-416]&quot; &quot;#,##0.00;[Red]&quot;-&quot;[$R$-416]&quot; &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="44" x14ac:knownFonts="1">
+  <fonts count="43" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -5782,14 +5803,6 @@
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <i/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
@@ -6131,9 +6144,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="173" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="167">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="10" applyProtection="1"/>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6296,10 +6309,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="169" fontId="29" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -6308,9 +6317,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="170" fontId="29" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -6339,7 +6345,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="30" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="171" fontId="24" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6368,61 +6374,61 @@
     <xf numFmtId="164" fontId="5" fillId="12" borderId="0" xfId="10" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="13" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="13" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="32" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="31" fillId="3" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="31" fillId="3" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="31" fillId="14" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="31" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="32" fillId="3" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="32" fillId="3" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="32" fillId="14" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="31" fillId="14" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="10" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="31" fillId="14" borderId="10" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="12" borderId="0" xfId="10" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -6446,7 +6452,7 @@
     <xf numFmtId="164" fontId="17" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="13" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6455,27 +6461,27 @@
     <xf numFmtId="164" fontId="16" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="36" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="38" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="37" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="35" fillId="5" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="34" fillId="5" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="36" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="165" fontId="5" fillId="8" borderId="1" xfId="10" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="37" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="36" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="31" fillId="6" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="30" fillId="6" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="24" fillId="6" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6493,14 +6499,14 @@
     <xf numFmtId="164" fontId="22" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="37" fillId="6" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="36" fillId="6" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="16" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="165" fontId="31" fillId="16" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="30" fillId="16" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="30" fillId="16" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="31" fillId="16" borderId="1" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="30" fillId="16" borderId="1" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="22" fillId="10" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6509,39 +6515,40 @@
     <xf numFmtId="165" fontId="26" fillId="12" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="40" fillId="6" borderId="1" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="39" fillId="6" borderId="1" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="26" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="31" fillId="3" borderId="1" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="168" fontId="30" fillId="3" borderId="1" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="168" fontId="21" fillId="6" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="41" fillId="3" borderId="1" xfId="16" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="40" fillId="3" borderId="1" xfId="16" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="41" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="42" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6551,18 +6558,17 @@
     <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -6576,34 +6582,34 @@
     <xf numFmtId="164" fontId="28" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="32" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="33" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="32" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="32" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="32" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="31" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="31" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="34" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="33" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6611,7 +6617,7 @@
     <xf numFmtId="164" fontId="16" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="34" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6626,13 +6632,13 @@
     <xf numFmtId="164" fontId="17" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="39" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="38" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6655,31 +6661,7 @@
     <cellStyle name="Result" xfId="14" xr:uid="{6F03FC13-A797-4115-B488-D5132E8D2E66}"/>
     <cellStyle name="Result2" xfId="15" xr:uid="{8B643F58-BFEA-4FDF-8CA6-D5886F8338D7}"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF8080"/>
-          <bgColor rgb="FFFF8080"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCCFFCC"/>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <font>
         <b/>
@@ -6709,6 +6691,42 @@
         <color rgb="FF666699"/>
         <family val="2"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF666699"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF8080"/>
+          <bgColor rgb="FFFF8080"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCFFCC"/>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -8532,18 +8550,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="140"/>
-      <c r="C1" s="140"/>
+      <c r="B1" s="133"/>
+      <c r="C1" s="133"/>
     </row>
     <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="134" t="s">
         <v>225</v>
       </c>
-      <c r="B2" s="141"/>
-      <c r="C2" s="141"/>
+      <c r="B2" s="134"/>
+      <c r="C2" s="134"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -8563,7 +8581,7 @@
       <c r="B4" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="C4" s="130" t="s">
+      <c r="C4" s="128" t="s">
         <v>220</v>
       </c>
     </row>
@@ -8574,7 +8592,7 @@
       <c r="B5" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C5" s="130" t="s">
+      <c r="C5" s="128" t="s">
         <v>223</v>
       </c>
     </row>
@@ -8585,7 +8603,7 @@
       <c r="B6" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C6" s="130" t="s">
+      <c r="C6" s="128" t="s">
         <v>224</v>
       </c>
     </row>
@@ -8681,38 +8699,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="139" t="s">
+      <c r="A1" s="137" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="F1" s="133" t="s">
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="F1" s="138" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="133"/>
-      <c r="H1" s="133"/>
-      <c r="I1" s="133"/>
-      <c r="J1" s="133"/>
-      <c r="K1" s="133"/>
-      <c r="L1" s="133"/>
+      <c r="G1" s="138"/>
+      <c r="H1" s="138"/>
+      <c r="I1" s="138"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="138"/>
+      <c r="L1" s="138"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="134" t="s">
+      <c r="A2" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="134"/>
-      <c r="C2" s="134"/>
-      <c r="D2" s="134"/>
-      <c r="F2" s="135" t="s">
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="F2" s="140" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="135"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -8733,20 +8751,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="136" t="s">
+      <c r="H3" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="136"/>
-      <c r="J3" s="136"/>
-      <c r="K3" s="136"/>
-      <c r="L3" s="136"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141"/>
+      <c r="K3" s="141"/>
+      <c r="L3" s="141"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="137" t="s">
+      <c r="A4" s="135" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="137"/>
-      <c r="C4" s="137"/>
+      <c r="B4" s="135"/>
+      <c r="C4" s="135"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -8789,7 +8807,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H5" s="15">
         <v>9</v>
@@ -8825,7 +8843,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H6" s="15">
         <v>9</v>
@@ -8861,7 +8879,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H7" s="15">
         <v>9</v>
@@ -8897,7 +8915,7 @@
         <v>4</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H8" s="15">
         <v>9</v>
@@ -8933,7 +8951,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H9" s="15">
         <v>9</v>
@@ -8977,11 +8995,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="137" t="s">
+      <c r="A11" s="135" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="137"/>
-      <c r="C11" s="137"/>
+      <c r="B11" s="135"/>
+      <c r="C11" s="135"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>49</v>
@@ -9076,8 +9094,8 @@
       <c r="B15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="132" t="s">
-        <v>230</v>
+      <c r="C15" s="130" t="s">
+        <v>228</v>
       </c>
       <c r="D15" s="13">
         <v>10</v>
@@ -9100,7 +9118,7 @@
       <c r="B16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="131" t="s">
+      <c r="C16" s="129" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="13">
@@ -9204,11 +9222,11 @@
       <c r="L20" s="21"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="137" t="s">
+      <c r="A21" s="135" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="137"/>
-      <c r="C21" s="137"/>
+      <c r="B21" s="135"/>
+      <c r="C21" s="135"/>
       <c r="D21" s="8">
         <f>SUM(D12:D20)</f>
         <v>53</v>
@@ -9246,7 +9264,7 @@
         <v>40</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D23" s="13">
         <v>10</v>
@@ -9260,7 +9278,7 @@
         <v>40</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D24" s="13">
         <v>10</v>
@@ -9274,7 +9292,7 @@
         <v>40</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D25" s="13">
         <v>10</v>
@@ -9288,7 +9306,7 @@
         <v>40</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D26" s="13">
         <v>10</v>
@@ -9302,7 +9320,7 @@
         <v>40</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D27" s="13">
         <v>10</v>
@@ -9316,7 +9334,7 @@
         <v>40</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D28" s="13">
         <v>10</v>
@@ -9330,7 +9348,7 @@
         <v>40</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="D29" s="13">
         <v>10</v>
@@ -9358,7 +9376,7 @@
         <v>40</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D31" s="13">
         <v>10</v>
@@ -9372,7 +9390,7 @@
         <v>40</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D32" s="13">
         <v>10</v>
@@ -9407,11 +9425,11 @@
       </c>
     </row>
     <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="137" t="s">
+      <c r="A35" s="135" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="137"/>
-      <c r="C35" s="137"/>
+      <c r="B35" s="135"/>
+      <c r="C35" s="135"/>
       <c r="D35" s="8">
         <f>SUM(D22:D34)</f>
         <v>104</v>
@@ -9544,9 +9562,9 @@
       </c>
     </row>
     <row r="45" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="138"/>
-      <c r="B45" s="138"/>
-      <c r="C45" s="138"/>
+      <c r="A45" s="136"/>
+      <c r="B45" s="136"/>
+      <c r="C45" s="136"/>
       <c r="D45" s="8">
         <f>SUM(D36:D44)</f>
         <v>34</v>
@@ -9560,16 +9578,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:L2"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -9592,19 +9610,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="142" t="s">
+      <c r="A1" s="131" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="142"/>
-      <c r="C1" s="142"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
     </row>
     <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="143" t="s">
+      <c r="A3" s="132" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="143"/>
-      <c r="C3" s="143"/>
+      <c r="B3" s="132"/>
+      <c r="C3" s="132"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
@@ -9669,7 +9687,7 @@
         <v>59</v>
       </c>
       <c r="B9" s="34">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="33" t="s">
         <v>60</v>
@@ -9711,11 +9729,11 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="143" t="s">
+      <c r="A14" s="132" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="143"/>
-      <c r="C14" s="143"/>
+      <c r="B14" s="132"/>
+      <c r="C14" s="132"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="s">
@@ -9811,9 +9829,9 @@
   <dimension ref="A1:AMJ16"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.125" style="74" customWidth="1"/>
+    <col min="1" max="1" width="6.125" style="72" customWidth="1"/>
     <col min="2" max="2" width="45.25" style="4" customWidth="1"/>
-    <col min="3" max="3" width="13.875" style="74" customWidth="1"/>
+    <col min="3" max="3" width="13.875" style="72" customWidth="1"/>
     <col min="4" max="6" width="13.125" style="4" customWidth="1"/>
     <col min="7" max="9" width="13" style="4" customWidth="1"/>
     <col min="10" max="10" width="13" style="23" customWidth="1"/>
@@ -9823,54 +9841,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="144" t="s">
+      <c r="A1" s="142" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="144"/>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="E1" s="144"/>
-      <c r="F1" s="144"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="144"/>
-      <c r="I1" s="144"/>
-      <c r="J1" s="144"/>
-      <c r="K1" s="144"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142"/>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
+      <c r="J1" s="142"/>
+      <c r="K1" s="142"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="145" t="s">
+      <c r="A2" s="143" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="145"/>
-      <c r="C2" s="145"/>
-      <c r="D2" s="145"/>
+      <c r="B2" s="143"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
       <c r="E2" s="44">
         <f>Planejamento!$B$10</f>
         <v>336</v>
       </c>
       <c r="F2" s="45"/>
-      <c r="G2" s="145" t="s">
+      <c r="G2" s="143" t="s">
         <v>76</v>
       </c>
-      <c r="H2" s="145"/>
-      <c r="I2" s="145"/>
-      <c r="J2" s="145"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
       <c r="K2" s="44"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="46"/>
       <c r="B3" s="47"/>
-      <c r="C3" s="146" t="s">
+      <c r="C3" s="144" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="146"/>
-      <c r="E3" s="146"/>
+      <c r="D3" s="144"/>
+      <c r="E3" s="144"/>
       <c r="F3" s="48"/>
-      <c r="G3" s="147" t="s">
+      <c r="G3" s="145" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="147"/>
-      <c r="I3" s="147"/>
+      <c r="H3" s="145"/>
+      <c r="I3" s="145"/>
       <c r="J3" s="50"/>
       <c r="K3" s="51"/>
     </row>
@@ -9913,208 +9931,254 @@
       <c r="A5" s="53">
         <v>1</v>
       </c>
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="60" t="s">
         <v>87</v>
       </c>
-      <c r="C5" s="55">
+      <c r="C5" s="61">
         <v>46092</v>
       </c>
-      <c r="D5" s="55">
+      <c r="D5" s="61">
         <v>46113</v>
       </c>
-      <c r="E5" s="56">
+      <c r="E5" s="62">
         <v>24</v>
       </c>
-      <c r="F5" s="57" t="s">
+      <c r="F5" s="63" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="55">
+      <c r="G5" s="54">
         <v>46092</v>
       </c>
-      <c r="H5" s="55">
-        <v>46118</v>
-      </c>
-      <c r="I5" s="56">
+      <c r="H5" s="54">
+        <v>46127</v>
+      </c>
+      <c r="I5" s="55">
         <v>28</v>
       </c>
-      <c r="J5" s="58">
+      <c r="J5" s="56">
         <f>E5-I5</f>
         <v>-4</v>
       </c>
-      <c r="K5" s="59" t="s">
+      <c r="K5" s="57" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A6" s="53">
         <v>2</v>
       </c>
-      <c r="B6" s="54" t="s">
-        <v>228</v>
-      </c>
-      <c r="C6" s="55">
+      <c r="B6" s="60" t="s">
+        <v>239</v>
+      </c>
+      <c r="C6" s="61">
         <v>46120</v>
       </c>
-      <c r="D6" s="55">
+      <c r="D6" s="61">
         <v>46127</v>
       </c>
-      <c r="E6" s="60">
-        <v>10</v>
-      </c>
-      <c r="F6" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="59"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E6" s="62">
+        <v>40</v>
+      </c>
+      <c r="F6" s="63" t="s">
+        <v>249</v>
+      </c>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="58"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="57"/>
+    </row>
+    <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="53">
         <v>3</v>
       </c>
-      <c r="B7" s="54" t="s">
-        <v>229</v>
-      </c>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="57" t="s">
+      <c r="B7" s="60" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="61">
+        <v>46127</v>
+      </c>
+      <c r="D7" s="61">
+        <v>46141</v>
+      </c>
+      <c r="E7" s="62">
+        <v>34</v>
+      </c>
+      <c r="F7" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="59"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G7" s="54"/>
+      <c r="H7" s="54"/>
+      <c r="I7" s="58"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="57"/>
+    </row>
+    <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A8" s="53">
         <v>4</v>
       </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="63"/>
-      <c r="D8" s="63"/>
-      <c r="E8" s="64"/>
-      <c r="F8" s="65"/>
-      <c r="G8" s="63"/>
-      <c r="H8" s="63"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="66"/>
-      <c r="K8" s="67"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="60" t="s">
+        <v>245</v>
+      </c>
+      <c r="C8" s="61">
+        <v>46141</v>
+      </c>
+      <c r="D8" s="61">
+        <v>46155</v>
+      </c>
+      <c r="E8" s="62">
+        <v>34</v>
+      </c>
+      <c r="F8" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="65"/>
+    </row>
+    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A9" s="53">
         <v>5</v>
       </c>
-      <c r="B9" s="62"/>
-      <c r="C9" s="63"/>
-      <c r="D9" s="63"/>
-      <c r="E9" s="64"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="63"/>
-      <c r="H9" s="63"/>
-      <c r="I9" s="64"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="67"/>
+      <c r="B9" s="60" t="s">
+        <v>246</v>
+      </c>
+      <c r="C9" s="61">
+        <v>46155</v>
+      </c>
+      <c r="D9" s="61">
+        <v>46534</v>
+      </c>
+      <c r="E9" s="62">
+        <v>34</v>
+      </c>
+      <c r="F9" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="61"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="65"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="53">
         <v>6</v>
       </c>
-      <c r="B10" s="62"/>
-      <c r="C10" s="63"/>
-      <c r="D10" s="63"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="65"/>
-      <c r="G10" s="63"/>
-      <c r="H10" s="63"/>
-      <c r="I10" s="64"/>
-      <c r="J10" s="66"/>
-      <c r="K10" s="67"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="60" t="s">
+        <v>247</v>
+      </c>
+      <c r="C10" s="61">
+        <v>46534</v>
+      </c>
+      <c r="D10" s="61">
+        <v>46548</v>
+      </c>
+      <c r="E10" s="62">
+        <v>34</v>
+      </c>
+      <c r="F10" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="65"/>
+    </row>
+    <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A11" s="53">
         <v>7</v>
       </c>
-      <c r="B11" s="62"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="64"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="63"/>
-      <c r="H11" s="63"/>
-      <c r="I11" s="64"/>
-      <c r="J11" s="66"/>
-      <c r="K11" s="67"/>
+      <c r="B11" s="60" t="s">
+        <v>248</v>
+      </c>
+      <c r="C11" s="61">
+        <v>46548</v>
+      </c>
+      <c r="D11" s="61">
+        <v>46197</v>
+      </c>
+      <c r="E11" s="62">
+        <v>34</v>
+      </c>
+      <c r="F11" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="64"/>
+      <c r="K11" s="65"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="53">
         <v>8</v>
       </c>
-      <c r="B12" s="62"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="64"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="63"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="66"/>
-      <c r="K12" s="67"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="62"/>
+      <c r="J12" s="64"/>
+      <c r="K12" s="65"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="53">
         <v>9</v>
       </c>
-      <c r="B13" s="62"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="65"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="63"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="66"/>
-      <c r="K13" s="67"/>
+      <c r="B13" s="60"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="61"/>
+      <c r="E13" s="62"/>
+      <c r="F13" s="63"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="62"/>
+      <c r="J13" s="64"/>
+      <c r="K13" s="65"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="53">
         <v>10</v>
       </c>
-      <c r="B14" s="62"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="65"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="63"/>
-      <c r="I14" s="64"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="67"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="63"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="62"/>
+      <c r="J14" s="64"/>
+      <c r="K14" s="65"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="68"/>
-      <c r="B15" s="69"/>
-      <c r="C15" s="70"/>
-      <c r="D15" s="69"/>
-      <c r="E15" s="71">
+      <c r="A15" s="66"/>
+      <c r="B15" s="67"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="69">
         <f>SUM(E5:E14)</f>
-        <v>34</v>
-      </c>
-      <c r="F15" s="69"/>
-      <c r="G15" s="72"/>
-      <c r="H15" s="72"/>
-      <c r="I15" s="71">
+        <v>234</v>
+      </c>
+      <c r="F15" s="67"/>
+      <c r="G15" s="70"/>
+      <c r="H15" s="70"/>
+      <c r="I15" s="69">
         <f>SUM(I5:I14)</f>
         <v>28</v>
       </c>
-      <c r="J15" s="73">
+      <c r="J15" s="71">
         <f>SUM(J5:J14)</f>
         <v>-4</v>
       </c>
-      <c r="K15" s="72"/>
+      <c r="K15" s="70"/>
     </row>
     <row r="16" spans="1:11" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="J16" s="23"/>
@@ -10128,29 +10192,29 @@
     <mergeCell ref="G3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:D14">
-    <cfRule type="expression" dxfId="9" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="8" stopIfTrue="1">
       <formula>OR($F5="Planned",$F5="Unplanned")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="9" stopIfTrue="1">
       <formula>$F5="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F14">
-    <cfRule type="expression" dxfId="7" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
       <formula>$F5="Planned"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
       <formula>$F5="Ongoing"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="5" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="5" stopIfTrue="1" operator="equal">
       <formula>"Unplanned"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:H14">
-    <cfRule type="expression" dxfId="4" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
       <formula>OR($F5="Planned",$F5="Unplanned")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
       <formula>$F5="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10170,615 +10234,637 @@
   <dimension ref="A1:AMJ60"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.625" style="76" customWidth="1"/>
-    <col min="2" max="2" width="35.625" style="76" customWidth="1"/>
-    <col min="3" max="3" width="6.5" style="76" customWidth="1"/>
-    <col min="4" max="4" width="13.25" style="76" customWidth="1"/>
-    <col min="5" max="5" width="8.875" style="76" customWidth="1"/>
-    <col min="6" max="6" width="12.5" style="76" customWidth="1"/>
-    <col min="7" max="7" width="9.125" style="76" customWidth="1"/>
-    <col min="8" max="9" width="12.25" style="76" customWidth="1"/>
-    <col min="10" max="10" width="24.25" style="76" customWidth="1"/>
-    <col min="11" max="11" width="27.875" style="76" customWidth="1"/>
-    <col min="12" max="12" width="8.5" style="76" customWidth="1"/>
-    <col min="13" max="14" width="20.5" style="76" customWidth="1"/>
-    <col min="15" max="256" width="8.5" style="76" customWidth="1"/>
-    <col min="257" max="258" width="6.5" style="76" customWidth="1"/>
-    <col min="259" max="259" width="13.875" style="76" customWidth="1"/>
-    <col min="260" max="260" width="9" style="76" customWidth="1"/>
-    <col min="261" max="261" width="13.5" style="76" customWidth="1"/>
-    <col min="262" max="262" width="10" style="76" customWidth="1"/>
-    <col min="263" max="263" width="12.25" style="76" customWidth="1"/>
-    <col min="264" max="264" width="5.875" style="76" customWidth="1"/>
-    <col min="265" max="265" width="24.25" style="76" customWidth="1"/>
-    <col min="266" max="266" width="32.5" style="76" customWidth="1"/>
-    <col min="267" max="267" width="17.625" style="76" customWidth="1"/>
-    <col min="268" max="268" width="8.5" style="76" customWidth="1"/>
-    <col min="269" max="270" width="20.5" style="76" customWidth="1"/>
-    <col min="271" max="512" width="8.5" style="76" customWidth="1"/>
-    <col min="513" max="514" width="6.5" style="76" customWidth="1"/>
-    <col min="515" max="515" width="13.875" style="76" customWidth="1"/>
-    <col min="516" max="516" width="9" style="76" customWidth="1"/>
-    <col min="517" max="517" width="13.5" style="76" customWidth="1"/>
-    <col min="518" max="518" width="10" style="76" customWidth="1"/>
-    <col min="519" max="519" width="12.25" style="76" customWidth="1"/>
-    <col min="520" max="520" width="5.875" style="76" customWidth="1"/>
-    <col min="521" max="521" width="24.25" style="76" customWidth="1"/>
-    <col min="522" max="522" width="32.5" style="76" customWidth="1"/>
-    <col min="523" max="523" width="17.625" style="76" customWidth="1"/>
-    <col min="524" max="524" width="8.5" style="76" customWidth="1"/>
-    <col min="525" max="526" width="20.5" style="76" customWidth="1"/>
-    <col min="527" max="768" width="8.5" style="76" customWidth="1"/>
-    <col min="769" max="770" width="6.5" style="76" customWidth="1"/>
-    <col min="771" max="771" width="13.875" style="76" customWidth="1"/>
-    <col min="772" max="772" width="9" style="76" customWidth="1"/>
-    <col min="773" max="773" width="13.5" style="76" customWidth="1"/>
-    <col min="774" max="774" width="10" style="76" customWidth="1"/>
-    <col min="775" max="775" width="12.25" style="76" customWidth="1"/>
-    <col min="776" max="776" width="5.875" style="76" customWidth="1"/>
-    <col min="777" max="777" width="24.25" style="76" customWidth="1"/>
-    <col min="778" max="778" width="32.5" style="76" customWidth="1"/>
-    <col min="779" max="779" width="17.625" style="76" customWidth="1"/>
-    <col min="780" max="780" width="8.5" style="76" customWidth="1"/>
-    <col min="781" max="782" width="20.5" style="76" customWidth="1"/>
-    <col min="783" max="1024" width="8.5" style="76" customWidth="1"/>
+    <col min="1" max="1" width="5.625" style="74" customWidth="1"/>
+    <col min="2" max="2" width="35.625" style="74" customWidth="1"/>
+    <col min="3" max="3" width="6.5" style="74" customWidth="1"/>
+    <col min="4" max="4" width="13.25" style="74" customWidth="1"/>
+    <col min="5" max="5" width="8.875" style="74" customWidth="1"/>
+    <col min="6" max="6" width="12.5" style="74" customWidth="1"/>
+    <col min="7" max="7" width="9.125" style="74" customWidth="1"/>
+    <col min="8" max="9" width="12.25" style="74" customWidth="1"/>
+    <col min="10" max="10" width="24.25" style="74" customWidth="1"/>
+    <col min="11" max="11" width="27.875" style="74" customWidth="1"/>
+    <col min="12" max="12" width="8.5" style="74" customWidth="1"/>
+    <col min="13" max="14" width="20.5" style="74" customWidth="1"/>
+    <col min="15" max="256" width="8.5" style="74" customWidth="1"/>
+    <col min="257" max="258" width="6.5" style="74" customWidth="1"/>
+    <col min="259" max="259" width="13.875" style="74" customWidth="1"/>
+    <col min="260" max="260" width="9" style="74" customWidth="1"/>
+    <col min="261" max="261" width="13.5" style="74" customWidth="1"/>
+    <col min="262" max="262" width="10" style="74" customWidth="1"/>
+    <col min="263" max="263" width="12.25" style="74" customWidth="1"/>
+    <col min="264" max="264" width="5.875" style="74" customWidth="1"/>
+    <col min="265" max="265" width="24.25" style="74" customWidth="1"/>
+    <col min="266" max="266" width="32.5" style="74" customWidth="1"/>
+    <col min="267" max="267" width="17.625" style="74" customWidth="1"/>
+    <col min="268" max="268" width="8.5" style="74" customWidth="1"/>
+    <col min="269" max="270" width="20.5" style="74" customWidth="1"/>
+    <col min="271" max="512" width="8.5" style="74" customWidth="1"/>
+    <col min="513" max="514" width="6.5" style="74" customWidth="1"/>
+    <col min="515" max="515" width="13.875" style="74" customWidth="1"/>
+    <col min="516" max="516" width="9" style="74" customWidth="1"/>
+    <col min="517" max="517" width="13.5" style="74" customWidth="1"/>
+    <col min="518" max="518" width="10" style="74" customWidth="1"/>
+    <col min="519" max="519" width="12.25" style="74" customWidth="1"/>
+    <col min="520" max="520" width="5.875" style="74" customWidth="1"/>
+    <col min="521" max="521" width="24.25" style="74" customWidth="1"/>
+    <col min="522" max="522" width="32.5" style="74" customWidth="1"/>
+    <col min="523" max="523" width="17.625" style="74" customWidth="1"/>
+    <col min="524" max="524" width="8.5" style="74" customWidth="1"/>
+    <col min="525" max="526" width="20.5" style="74" customWidth="1"/>
+    <col min="527" max="768" width="8.5" style="74" customWidth="1"/>
+    <col min="769" max="770" width="6.5" style="74" customWidth="1"/>
+    <col min="771" max="771" width="13.875" style="74" customWidth="1"/>
+    <col min="772" max="772" width="9" style="74" customWidth="1"/>
+    <col min="773" max="773" width="13.5" style="74" customWidth="1"/>
+    <col min="774" max="774" width="10" style="74" customWidth="1"/>
+    <col min="775" max="775" width="12.25" style="74" customWidth="1"/>
+    <col min="776" max="776" width="5.875" style="74" customWidth="1"/>
+    <col min="777" max="777" width="24.25" style="74" customWidth="1"/>
+    <col min="778" max="778" width="32.5" style="74" customWidth="1"/>
+    <col min="779" max="779" width="17.625" style="74" customWidth="1"/>
+    <col min="780" max="780" width="8.5" style="74" customWidth="1"/>
+    <col min="781" max="782" width="20.5" style="74" customWidth="1"/>
+    <col min="783" max="1024" width="8.5" style="74" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="75" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="144" t="s">
+    <row r="1" spans="1:11" s="73" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="142" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="144"/>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="E1" s="144"/>
-      <c r="F1" s="144"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="144"/>
-      <c r="I1" s="144"/>
-      <c r="J1" s="144"/>
-      <c r="K1" s="144"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142"/>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
+      <c r="J1" s="142"/>
+      <c r="K1" s="142"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D3" s="77" t="s">
+      <c r="D3" s="75" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D4" s="78" t="s">
+      <c r="D4" s="76" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D5" s="78" t="s">
+      <c r="D5" s="76" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D6" s="78" t="s">
+      <c r="D6" s="76" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D7" s="78" t="s">
+      <c r="D7" s="76" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D8" s="78" t="s">
+      <c r="D8" s="76" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D9" s="78" t="s">
+      <c r="D9" s="76" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D10" s="78" t="s">
+      <c r="D10" s="76" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D11" s="78" t="s">
+      <c r="D11" s="76" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D12" s="78" t="s">
+      <c r="D12" s="76" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D13" s="78" t="s">
+      <c r="D13" s="76" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D14" s="77" t="s">
+      <c r="D14" s="75" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D15" s="78" t="s">
+      <c r="D15" s="76" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D16" s="78" t="s">
+      <c r="D16" s="76" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="17" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D17" s="78" t="s">
+      <c r="D17" s="76" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="18" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D18" s="77" t="s">
+      <c r="D18" s="75" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="19" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D19" s="78" t="s">
+      <c r="D19" s="76" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="20" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D20" s="78" t="s">
+      <c r="D20" s="76" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D21" s="78" t="s">
+      <c r="D21" s="76" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D22" s="77" t="s">
+      <c r="D22" s="75" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D23" s="78" t="s">
+      <c r="D23" s="76" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="24" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D24" s="78" t="s">
+      <c r="D24" s="76" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="25" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D25" s="78" t="s">
+      <c r="D25" s="76" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="26" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D26" s="78" t="s">
+      <c r="D26" s="76" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="27" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D27" s="77" t="s">
+      <c r="D27" s="75" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="28" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D28" s="78" t="s">
+      <c r="D28" s="76" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="29" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D29" s="78" t="s">
+      <c r="D29" s="76" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="30" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D30" s="78" t="s">
+      <c r="D30" s="76" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="4:4" s="79" customFormat="1" ht="11.25" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D31" s="80" t="s">
+    <row r="31" spans="4:4" s="77" customFormat="1" ht="11.25" hidden="1" x14ac:dyDescent="0.2">
+      <c r="D31" s="78" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="32" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D32" s="81" t="s">
+      <c r="D32" s="79" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D33" s="149" t="s">
+      <c r="D33" s="153" t="s">
         <v>122</v>
       </c>
-      <c r="E33" s="149"/>
+      <c r="E33" s="153"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D34" s="78">
+      <c r="D34" s="76">
         <v>4290</v>
       </c>
-      <c r="E34" s="78" t="s">
+      <c r="E34" s="76" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D35" s="78">
+      <c r="D35" s="76">
         <v>5082</v>
       </c>
-      <c r="E35" s="78" t="s">
+      <c r="E35" s="76" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D36" s="78">
+      <c r="D36" s="76">
         <v>4356</v>
       </c>
-      <c r="E36" s="78" t="s">
+      <c r="E36" s="76" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D37" s="78">
+      <c r="D37" s="76">
         <v>5929</v>
       </c>
-      <c r="E37" s="78" t="s">
+      <c r="E37" s="76" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D38" s="78">
+      <c r="D38" s="76">
         <v>5005</v>
       </c>
-      <c r="E38" s="78" t="s">
+      <c r="E38" s="76" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D39" s="78">
+      <c r="D39" s="76">
         <v>4225</v>
       </c>
-      <c r="E39" s="78" t="s">
+      <c r="E39" s="76" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:11" s="75" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="150" t="s">
+    <row r="41" spans="1:11" s="73" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="154" t="s">
         <v>129</v>
       </c>
-      <c r="B41" s="150"/>
-      <c r="C41" s="150"/>
-      <c r="D41" s="150"/>
-      <c r="E41" s="150"/>
-      <c r="F41" s="150"/>
-      <c r="G41" s="150"/>
-      <c r="H41" s="150"/>
-      <c r="I41" s="150"/>
-      <c r="J41" s="150"/>
-      <c r="K41" s="150"/>
-    </row>
-    <row r="42" spans="1:11" s="75" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="151" t="s">
+      <c r="B41" s="154"/>
+      <c r="C41" s="154"/>
+      <c r="D41" s="154"/>
+      <c r="E41" s="154"/>
+      <c r="F41" s="154"/>
+      <c r="G41" s="154"/>
+      <c r="H41" s="154"/>
+      <c r="I41" s="154"/>
+      <c r="J41" s="154"/>
+      <c r="K41" s="154"/>
+    </row>
+    <row r="42" spans="1:11" s="73" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="155" t="s">
         <v>130</v>
       </c>
-      <c r="B42" s="151"/>
-      <c r="C42" s="151"/>
-      <c r="D42" s="151"/>
-      <c r="E42" s="151"/>
-      <c r="F42" s="151"/>
-      <c r="G42" s="151"/>
-      <c r="H42" s="151"/>
-      <c r="I42" s="151"/>
-      <c r="J42" s="151"/>
-      <c r="K42" s="151"/>
-    </row>
-    <row r="43" spans="1:11" s="75" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="152" t="s">
+      <c r="B42" s="155"/>
+      <c r="C42" s="155"/>
+      <c r="D42" s="155"/>
+      <c r="E42" s="155"/>
+      <c r="F42" s="155"/>
+      <c r="G42" s="155"/>
+      <c r="H42" s="155"/>
+      <c r="I42" s="155"/>
+      <c r="J42" s="155"/>
+      <c r="K42" s="155"/>
+    </row>
+    <row r="43" spans="1:11" s="73" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="156" t="s">
         <v>131</v>
       </c>
-      <c r="B43" s="152"/>
-      <c r="C43" s="152"/>
-      <c r="D43" s="152"/>
-      <c r="E43" s="152"/>
-      <c r="F43" s="152"/>
-      <c r="G43" s="152"/>
-      <c r="H43" s="152"/>
-      <c r="I43" s="152"/>
-      <c r="J43" s="152"/>
-      <c r="K43" s="152"/>
-    </row>
-    <row r="44" spans="1:11" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="148" t="s">
+      <c r="B43" s="156"/>
+      <c r="C43" s="156"/>
+      <c r="D43" s="156"/>
+      <c r="E43" s="156"/>
+      <c r="F43" s="156"/>
+      <c r="G43" s="156"/>
+      <c r="H43" s="156"/>
+      <c r="I43" s="156"/>
+      <c r="J43" s="156"/>
+      <c r="K43" s="156"/>
+    </row>
+    <row r="44" spans="1:11" s="73" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="152" t="s">
         <v>132</v>
       </c>
-      <c r="B44" s="148"/>
-      <c r="C44" s="148"/>
-      <c r="D44" s="148"/>
-      <c r="E44" s="148"/>
-      <c r="F44" s="148"/>
-      <c r="G44" s="148"/>
-      <c r="H44" s="148"/>
-      <c r="I44" s="148"/>
-      <c r="J44" s="148"/>
-      <c r="K44" s="148"/>
+      <c r="B44" s="152"/>
+      <c r="C44" s="152"/>
+      <c r="D44" s="152"/>
+      <c r="E44" s="152"/>
+      <c r="F44" s="152"/>
+      <c r="G44" s="152"/>
+      <c r="H44" s="152"/>
+      <c r="I44" s="152"/>
+      <c r="J44" s="152"/>
+      <c r="K44" s="152"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="155" t="s">
+      <c r="A46" s="148" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="155"/>
-      <c r="C46" s="155"/>
-      <c r="D46" s="155"/>
-      <c r="E46" s="155"/>
-      <c r="F46" s="155"/>
-      <c r="G46" s="155"/>
-      <c r="H46" s="155"/>
-      <c r="I46" s="155"/>
-      <c r="J46" s="155"/>
-      <c r="K46" s="155"/>
-    </row>
-    <row r="47" spans="1:11" s="84" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="82" t="s">
+      <c r="B46" s="148"/>
+      <c r="C46" s="148"/>
+      <c r="D46" s="148"/>
+      <c r="E46" s="148"/>
+      <c r="F46" s="148"/>
+      <c r="G46" s="148"/>
+      <c r="H46" s="148"/>
+      <c r="I46" s="148"/>
+      <c r="J46" s="148"/>
+      <c r="K46" s="148"/>
+    </row>
+    <row r="47" spans="1:11" s="82" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="80" t="s">
         <v>134</v>
       </c>
-      <c r="B47" s="83"/>
-      <c r="C47" s="156" t="s">
+      <c r="B47" s="81"/>
+      <c r="C47" s="149" t="s">
         <v>135</v>
       </c>
-      <c r="D47" s="156"/>
-      <c r="E47" s="156"/>
-      <c r="F47" s="156"/>
-      <c r="G47" s="156"/>
-      <c r="H47" s="156"/>
-      <c r="I47" s="156"/>
-      <c r="J47" s="156"/>
-      <c r="K47" s="156"/>
-    </row>
-    <row r="48" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="157"/>
-      <c r="B48" s="153" t="s">
+      <c r="D47" s="149"/>
+      <c r="E47" s="149"/>
+      <c r="F47" s="149"/>
+      <c r="G47" s="149"/>
+      <c r="H47" s="149"/>
+      <c r="I47" s="149"/>
+      <c r="J47" s="149"/>
+      <c r="K47" s="149"/>
+    </row>
+    <row r="48" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="150"/>
+      <c r="B48" s="146" t="s">
         <v>136</v>
       </c>
-      <c r="C48" s="153" t="s">
+      <c r="C48" s="146" t="s">
         <v>137</v>
       </c>
-      <c r="D48" s="153" t="s">
+      <c r="D48" s="146" t="s">
         <v>138</v>
       </c>
-      <c r="E48" s="153" t="s">
+      <c r="E48" s="146" t="s">
         <v>107</v>
       </c>
-      <c r="F48" s="153" t="s">
+      <c r="F48" s="146" t="s">
         <v>139</v>
       </c>
-      <c r="G48" s="153" t="s">
+      <c r="G48" s="146" t="s">
         <v>111</v>
       </c>
-      <c r="H48" s="158" t="s">
+      <c r="H48" s="151" t="s">
         <v>140</v>
       </c>
-      <c r="I48" s="158"/>
-      <c r="J48" s="158"/>
-      <c r="K48" s="158"/>
-    </row>
-    <row r="49" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="157"/>
-      <c r="B49" s="153"/>
-      <c r="C49" s="153"/>
-      <c r="D49" s="153"/>
-      <c r="E49" s="153"/>
-      <c r="F49" s="153"/>
-      <c r="G49" s="153"/>
-      <c r="H49" s="153" t="s">
+      <c r="I48" s="151"/>
+      <c r="J48" s="151"/>
+      <c r="K48" s="151"/>
+    </row>
+    <row r="49" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="150"/>
+      <c r="B49" s="146"/>
+      <c r="C49" s="146"/>
+      <c r="D49" s="146"/>
+      <c r="E49" s="146"/>
+      <c r="F49" s="146"/>
+      <c r="G49" s="146"/>
+      <c r="H49" s="146" t="s">
         <v>141</v>
       </c>
-      <c r="I49" s="153"/>
-      <c r="J49" s="85" t="s">
+      <c r="I49" s="146"/>
+      <c r="J49" s="83" t="s">
         <v>142</v>
       </c>
-      <c r="K49" s="85" t="s">
+      <c r="K49" s="83" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="50" spans="1:11" s="86" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="87">
+    <row r="50" spans="1:11" s="84" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="85">
         <v>1</v>
       </c>
-      <c r="B50" s="88" t="s">
+      <c r="B50" s="86" t="s">
         <v>144</v>
       </c>
-      <c r="C50" s="89">
-        <v>46184</v>
-      </c>
-      <c r="D50" s="90" t="s">
+      <c r="C50" s="87">
+        <v>46092</v>
+      </c>
+      <c r="D50" s="88" t="s">
         <v>104</v>
       </c>
-      <c r="E50" s="90" t="s">
+      <c r="E50" s="88" t="s">
         <v>109</v>
       </c>
-      <c r="F50" s="91" t="str">
+      <c r="F50" s="89" t="str">
         <f t="shared" ref="F50:F60" si="0">IF(OR((CODE($D50)*CODE($E50))=$D$36,(CODE($D50)*CODE($E50))=$D$35),$D$15,IF(OR((CODE($D50)*CODE($E50))=$D$34,(CODE($D50)*CODE($E50))=$D$37),$D$16,IF(OR((CODE($D50)*CODE($E50))=$D$38,(CODE($D50)*CODE($E50))=$D$39),$D$17,0)))</f>
         <v>Baixa</v>
       </c>
-      <c r="G50" s="90" t="s">
+      <c r="G50" s="88" t="s">
         <v>112</v>
       </c>
-      <c r="H50" s="154"/>
-      <c r="I50" s="154"/>
-      <c r="J50" s="92" t="s">
+      <c r="H50" s="147"/>
+      <c r="I50" s="147"/>
+      <c r="J50" s="90" t="s">
         <v>227</v>
       </c>
-      <c r="K50" s="92" t="s">
+      <c r="K50" s="90" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="51" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="87"/>
-      <c r="B51" s="88"/>
-      <c r="C51" s="89"/>
-      <c r="D51" s="90"/>
-      <c r="E51" s="90"/>
-      <c r="F51" s="91" t="e">
+    <row r="51" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="85">
+        <v>2</v>
+      </c>
+      <c r="B51" s="86" t="s">
+        <v>250</v>
+      </c>
+      <c r="C51" s="87">
+        <v>46123</v>
+      </c>
+      <c r="D51" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="E51" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="F51" s="89" t="str">
+        <f t="shared" si="0"/>
+        <v>Alta</v>
+      </c>
+      <c r="G51" s="88" t="s">
+        <v>112</v>
+      </c>
+      <c r="H51" s="91"/>
+      <c r="I51" s="92"/>
+      <c r="J51" s="90" t="s">
+        <v>251</v>
+      </c>
+      <c r="K51" s="90" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="85"/>
+      <c r="B52" s="86"/>
+      <c r="C52" s="87"/>
+      <c r="D52" s="88"/>
+      <c r="E52" s="88"/>
+      <c r="F52" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G51" s="90"/>
-      <c r="H51" s="93"/>
-      <c r="I51" s="94"/>
-      <c r="J51" s="92"/>
-      <c r="K51" s="92"/>
-    </row>
-    <row r="52" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="87"/>
-      <c r="B52" s="88"/>
-      <c r="C52" s="89"/>
-      <c r="D52" s="90"/>
-      <c r="E52" s="90"/>
-      <c r="F52" s="91" t="e">
+      <c r="G52" s="88"/>
+      <c r="H52" s="91"/>
+      <c r="I52" s="92"/>
+      <c r="J52" s="90"/>
+      <c r="K52" s="90"/>
+    </row>
+    <row r="53" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="85"/>
+      <c r="B53" s="86"/>
+      <c r="C53" s="87"/>
+      <c r="D53" s="88"/>
+      <c r="E53" s="88"/>
+      <c r="F53" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G52" s="90"/>
-      <c r="H52" s="93"/>
-      <c r="I52" s="94"/>
-      <c r="J52" s="92"/>
-      <c r="K52" s="92"/>
-    </row>
-    <row r="53" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="87"/>
-      <c r="B53" s="88"/>
-      <c r="C53" s="89"/>
-      <c r="D53" s="90"/>
-      <c r="E53" s="90"/>
-      <c r="F53" s="91" t="e">
+      <c r="G53" s="88"/>
+      <c r="H53" s="91"/>
+      <c r="I53" s="92"/>
+      <c r="J53" s="90"/>
+      <c r="K53" s="90"/>
+    </row>
+    <row r="54" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="85"/>
+      <c r="B54" s="86"/>
+      <c r="C54" s="87"/>
+      <c r="D54" s="88"/>
+      <c r="E54" s="88"/>
+      <c r="F54" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G53" s="90"/>
-      <c r="H53" s="93"/>
-      <c r="I53" s="94"/>
-      <c r="J53" s="92"/>
-      <c r="K53" s="92"/>
-    </row>
-    <row r="54" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="87"/>
-      <c r="B54" s="88"/>
-      <c r="C54" s="89"/>
-      <c r="D54" s="90"/>
-      <c r="E54" s="90"/>
-      <c r="F54" s="91" t="e">
+      <c r="G54" s="88"/>
+      <c r="H54" s="91"/>
+      <c r="I54" s="92"/>
+      <c r="J54" s="90"/>
+      <c r="K54" s="90"/>
+    </row>
+    <row r="55" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="85"/>
+      <c r="B55" s="86"/>
+      <c r="C55" s="87"/>
+      <c r="D55" s="88"/>
+      <c r="E55" s="88"/>
+      <c r="F55" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G54" s="90"/>
-      <c r="H54" s="93"/>
-      <c r="I54" s="94"/>
-      <c r="J54" s="92"/>
-      <c r="K54" s="92"/>
-    </row>
-    <row r="55" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="87"/>
-      <c r="B55" s="88"/>
-      <c r="C55" s="89"/>
-      <c r="D55" s="90"/>
-      <c r="E55" s="90"/>
-      <c r="F55" s="91" t="e">
+      <c r="G55" s="88"/>
+      <c r="H55" s="91"/>
+      <c r="I55" s="92"/>
+      <c r="J55" s="90"/>
+      <c r="K55" s="90"/>
+    </row>
+    <row r="56" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="85"/>
+      <c r="B56" s="86"/>
+      <c r="C56" s="87"/>
+      <c r="D56" s="88"/>
+      <c r="E56" s="88"/>
+      <c r="F56" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G55" s="90"/>
-      <c r="H55" s="93"/>
-      <c r="I55" s="94"/>
-      <c r="J55" s="92"/>
-      <c r="K55" s="92"/>
-    </row>
-    <row r="56" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="87"/>
-      <c r="B56" s="88"/>
-      <c r="C56" s="89"/>
-      <c r="D56" s="90"/>
-      <c r="E56" s="90"/>
-      <c r="F56" s="91" t="e">
+      <c r="G56" s="88"/>
+      <c r="H56" s="91"/>
+      <c r="I56" s="92"/>
+      <c r="J56" s="90"/>
+      <c r="K56" s="90"/>
+    </row>
+    <row r="57" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="85"/>
+      <c r="B57" s="86"/>
+      <c r="C57" s="87"/>
+      <c r="D57" s="88"/>
+      <c r="E57" s="88"/>
+      <c r="F57" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G56" s="90"/>
-      <c r="H56" s="93"/>
-      <c r="I56" s="94"/>
-      <c r="J56" s="92"/>
-      <c r="K56" s="92"/>
-    </row>
-    <row r="57" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="87"/>
-      <c r="B57" s="88"/>
-      <c r="C57" s="89"/>
-      <c r="D57" s="90"/>
-      <c r="E57" s="90"/>
-      <c r="F57" s="91" t="e">
+      <c r="G57" s="88"/>
+      <c r="H57" s="91"/>
+      <c r="I57" s="92"/>
+      <c r="J57" s="90"/>
+      <c r="K57" s="90"/>
+    </row>
+    <row r="58" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="85"/>
+      <c r="B58" s="86"/>
+      <c r="C58" s="87"/>
+      <c r="D58" s="88"/>
+      <c r="E58" s="88"/>
+      <c r="F58" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G57" s="90"/>
-      <c r="H57" s="93"/>
-      <c r="I57" s="94"/>
-      <c r="J57" s="92"/>
-      <c r="K57" s="92"/>
-    </row>
-    <row r="58" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="87"/>
-      <c r="B58" s="88"/>
-      <c r="C58" s="89"/>
-      <c r="D58" s="90"/>
-      <c r="E58" s="90"/>
-      <c r="F58" s="91" t="e">
+      <c r="G58" s="88"/>
+      <c r="H58" s="91"/>
+      <c r="I58" s="92"/>
+      <c r="J58" s="90"/>
+      <c r="K58" s="90"/>
+    </row>
+    <row r="59" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="85"/>
+      <c r="B59" s="86"/>
+      <c r="C59" s="87"/>
+      <c r="D59" s="88"/>
+      <c r="E59" s="88"/>
+      <c r="F59" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G58" s="90"/>
-      <c r="H58" s="93"/>
-      <c r="I58" s="94"/>
-      <c r="J58" s="92"/>
-      <c r="K58" s="92"/>
-    </row>
-    <row r="59" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="87"/>
-      <c r="B59" s="88"/>
-      <c r="C59" s="89"/>
-      <c r="D59" s="90"/>
-      <c r="E59" s="90"/>
-      <c r="F59" s="91" t="e">
+      <c r="G59" s="88"/>
+      <c r="H59" s="147"/>
+      <c r="I59" s="147"/>
+      <c r="J59" s="90"/>
+      <c r="K59" s="90"/>
+    </row>
+    <row r="60" spans="1:11" s="84" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="85"/>
+      <c r="B60" s="86"/>
+      <c r="C60" s="87"/>
+      <c r="D60" s="88"/>
+      <c r="E60" s="88"/>
+      <c r="F60" s="89" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="G59" s="90"/>
-      <c r="H59" s="154"/>
-      <c r="I59" s="154"/>
-      <c r="J59" s="92"/>
-      <c r="K59" s="92"/>
-    </row>
-    <row r="60" spans="1:11" s="86" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="87"/>
-      <c r="B60" s="88"/>
-      <c r="C60" s="89"/>
-      <c r="D60" s="90"/>
-      <c r="E60" s="90"/>
-      <c r="F60" s="91" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G60" s="90"/>
-      <c r="H60" s="154"/>
-      <c r="I60" s="154"/>
-      <c r="J60" s="92"/>
-      <c r="K60" s="92"/>
+      <c r="G60" s="88"/>
+      <c r="H60" s="147"/>
+      <c r="I60" s="147"/>
+      <c r="J60" s="90"/>
+      <c r="K60" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -10793,21 +10879,15 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
-    <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="8" stopIfTrue="1" operator="equal">
       <formula>$D$15</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="9" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="9" stopIfTrue="1" operator="equal">
       <formula>$D$16</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="10" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="10" stopIfTrue="1" operator="equal">
       <formula>$D$17</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10855,432 +10935,432 @@
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="75" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="161" t="s">
+    <row r="1" spans="1:23" s="73" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="159" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="161"/>
-      <c r="E1" s="161"/>
-      <c r="F1" s="161"/>
-      <c r="G1" s="161"/>
-      <c r="H1" s="161"/>
-      <c r="I1" s="161"/>
-      <c r="J1" s="161"/>
-      <c r="K1" s="161"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="161"/>
-    </row>
-    <row r="2" spans="1:23" s="95" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="162" t="s">
+      <c r="B1" s="159"/>
+      <c r="C1" s="159"/>
+      <c r="D1" s="159"/>
+      <c r="E1" s="159"/>
+      <c r="F1" s="159"/>
+      <c r="G1" s="159"/>
+      <c r="H1" s="159"/>
+      <c r="I1" s="159"/>
+      <c r="J1" s="159"/>
+      <c r="K1" s="159"/>
+      <c r="L1" s="159"/>
+      <c r="M1" s="159"/>
+      <c r="N1" s="159"/>
+    </row>
+    <row r="2" spans="1:23" s="93" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="160" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="162"/>
-      <c r="C2" s="162"/>
-      <c r="D2" s="162"/>
-      <c r="E2" s="162"/>
-      <c r="F2" s="162"/>
-      <c r="G2" s="162"/>
-      <c r="H2" s="162"/>
-      <c r="I2" s="162"/>
-      <c r="J2" s="162"/>
-      <c r="K2" s="162"/>
-      <c r="L2" s="162"/>
-      <c r="M2" s="162"/>
-      <c r="N2" s="162"/>
-    </row>
-    <row r="3" spans="1:23" s="95" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="163" t="s">
+      <c r="B2" s="160"/>
+      <c r="C2" s="160"/>
+      <c r="D2" s="160"/>
+      <c r="E2" s="160"/>
+      <c r="F2" s="160"/>
+      <c r="G2" s="160"/>
+      <c r="H2" s="160"/>
+      <c r="I2" s="160"/>
+      <c r="J2" s="160"/>
+      <c r="K2" s="160"/>
+      <c r="L2" s="160"/>
+      <c r="M2" s="160"/>
+      <c r="N2" s="160"/>
+    </row>
+    <row r="3" spans="1:23" s="93" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="161" t="s">
         <v>146</v>
       </c>
-      <c r="B3" s="163"/>
-      <c r="C3" s="163"/>
-      <c r="D3" s="163"/>
-      <c r="E3" s="163"/>
-      <c r="F3" s="163"/>
-      <c r="G3" s="163"/>
-      <c r="H3" s="163"/>
-      <c r="I3" s="163"/>
-      <c r="J3" s="163"/>
-      <c r="K3" s="163"/>
-      <c r="L3" s="163"/>
-      <c r="M3" s="163"/>
-      <c r="N3" s="163"/>
-    </row>
-    <row r="4" spans="1:23" s="95" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="164" t="s">
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="161"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
+    </row>
+    <row r="4" spans="1:23" s="93" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="162" t="s">
         <v>147</v>
       </c>
-      <c r="B4" s="164"/>
-      <c r="C4" s="164"/>
-      <c r="D4" s="164"/>
-      <c r="E4" s="164"/>
-      <c r="F4" s="164"/>
-      <c r="G4" s="164"/>
-      <c r="H4" s="164"/>
-      <c r="I4" s="164"/>
-      <c r="J4" s="164"/>
-      <c r="K4" s="164"/>
-      <c r="L4" s="164"/>
-      <c r="M4" s="164"/>
-      <c r="N4" s="164"/>
-    </row>
-    <row r="5" spans="1:23" s="95" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="165" t="s">
+      <c r="B4" s="162"/>
+      <c r="C4" s="162"/>
+      <c r="D4" s="162"/>
+      <c r="E4" s="162"/>
+      <c r="F4" s="162"/>
+      <c r="G4" s="162"/>
+      <c r="H4" s="162"/>
+      <c r="I4" s="162"/>
+      <c r="J4" s="162"/>
+      <c r="K4" s="162"/>
+      <c r="L4" s="162"/>
+      <c r="M4" s="162"/>
+      <c r="N4" s="162"/>
+    </row>
+    <row r="5" spans="1:23" s="93" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="163" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="165"/>
-      <c r="C5" s="165"/>
-      <c r="D5" s="165"/>
-      <c r="E5" s="165"/>
-      <c r="F5" s="165"/>
-      <c r="G5" s="165"/>
-      <c r="H5" s="165"/>
-      <c r="I5" s="165"/>
-      <c r="J5" s="165"/>
-      <c r="K5" s="165"/>
-      <c r="L5" s="165"/>
-      <c r="M5" s="165"/>
-      <c r="N5" s="165"/>
+      <c r="B5" s="163"/>
+      <c r="C5" s="163"/>
+      <c r="D5" s="163"/>
+      <c r="E5" s="163"/>
+      <c r="F5" s="163"/>
+      <c r="G5" s="163"/>
+      <c r="H5" s="163"/>
+      <c r="I5" s="163"/>
+      <c r="J5" s="163"/>
+      <c r="K5" s="163"/>
+      <c r="L5" s="163"/>
+      <c r="M5" s="163"/>
+      <c r="N5" s="163"/>
     </row>
     <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="159" t="s">
+      <c r="A7" s="157" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="159"/>
-      <c r="D7" s="159" t="s">
+      <c r="B7" s="157"/>
+      <c r="D7" s="157" t="s">
         <v>150</v>
       </c>
-      <c r="E7" s="159"/>
-      <c r="G7" s="159" t="s">
+      <c r="E7" s="157"/>
+      <c r="G7" s="157" t="s">
         <v>151</v>
       </c>
-      <c r="H7" s="159"/>
-      <c r="I7" s="159"/>
-      <c r="J7" s="159"/>
-      <c r="K7" s="159"/>
-      <c r="M7" s="159" t="s">
+      <c r="H7" s="157"/>
+      <c r="I7" s="157"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="157"/>
+      <c r="M7" s="157" t="s">
         <v>152</v>
       </c>
-      <c r="N7" s="159"/>
+      <c r="N7" s="157"/>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="98" t="s">
+      <c r="A8" s="96" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="99" t="s">
+      <c r="B8" s="97" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="98" t="s">
+      <c r="D8" s="96" t="s">
         <v>155</v>
       </c>
-      <c r="E8" s="99" t="s">
+      <c r="E8" s="97" t="s">
         <v>154</v>
       </c>
-      <c r="G8" s="98" t="s">
+      <c r="G8" s="96" t="s">
         <v>156</v>
       </c>
-      <c r="H8" s="98" t="s">
+      <c r="H8" s="96" t="s">
         <v>157</v>
       </c>
-      <c r="I8" s="98" t="s">
+      <c r="I8" s="96" t="s">
         <v>105</v>
       </c>
-      <c r="J8" s="99" t="s">
+      <c r="J8" s="97" t="s">
         <v>158</v>
       </c>
-      <c r="K8" s="99" t="s">
+      <c r="K8" s="97" t="s">
         <v>159</v>
       </c>
-      <c r="M8" s="99" t="s">
+      <c r="M8" s="97" t="s">
         <v>160</v>
       </c>
-      <c r="N8" s="99" t="s">
+      <c r="N8" s="97" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A9" s="96" t="s">
+      <c r="A9" s="94" t="s">
         <v>162</v>
       </c>
-      <c r="B9" s="97" t="s">
+      <c r="B9" s="95" t="s">
         <v>157</v>
       </c>
-      <c r="D9" s="96" t="s">
+      <c r="D9" s="94" t="s">
         <v>163</v>
       </c>
-      <c r="E9" s="97" t="s">
+      <c r="E9" s="95" t="s">
         <v>157</v>
       </c>
-      <c r="G9" s="98" t="s">
+      <c r="G9" s="96" t="s">
         <v>164</v>
       </c>
-      <c r="H9" s="96">
+      <c r="H9" s="94">
         <v>2</v>
       </c>
-      <c r="I9" s="96">
+      <c r="I9" s="94">
         <v>0</v>
       </c>
-      <c r="J9" s="96">
+      <c r="J9" s="94">
         <v>0</v>
       </c>
-      <c r="K9" s="99">
+      <c r="K9" s="97">
         <f>(H9*4)+(I9*6)+(J9*8)</f>
         <v>8</v>
       </c>
-      <c r="M9" s="100" t="s">
+      <c r="M9" s="98" t="s">
         <v>165</v>
       </c>
-      <c r="N9" s="101"/>
+      <c r="N9" s="99"/>
     </row>
     <row r="10" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A10" s="96" t="s">
+      <c r="A10" s="94" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="97" t="s">
+      <c r="B10" s="95" t="s">
         <v>157</v>
       </c>
-      <c r="D10" s="96"/>
-      <c r="E10" s="97"/>
-      <c r="G10" s="98" t="s">
+      <c r="D10" s="94"/>
+      <c r="E10" s="95"/>
+      <c r="G10" s="96" t="s">
         <v>167</v>
       </c>
-      <c r="H10" s="96"/>
-      <c r="I10" s="96"/>
-      <c r="J10" s="96"/>
-      <c r="K10" s="99">
+      <c r="H10" s="94"/>
+      <c r="I10" s="94"/>
+      <c r="J10" s="94"/>
+      <c r="K10" s="97">
         <f>(H10*3)+(I10*4)+(J10*6)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="100" t="s">
+      <c r="M10" s="98" t="s">
         <v>168</v>
       </c>
-      <c r="N10" s="101"/>
+      <c r="N10" s="99"/>
     </row>
     <row r="11" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="96"/>
-      <c r="B11" s="97"/>
-      <c r="D11" s="96"/>
-      <c r="E11" s="97"/>
-      <c r="G11" s="159" t="s">
+      <c r="A11" s="94"/>
+      <c r="B11" s="95"/>
+      <c r="D11" s="94"/>
+      <c r="E11" s="95"/>
+      <c r="G11" s="157" t="s">
         <v>169</v>
       </c>
-      <c r="H11" s="159"/>
-      <c r="I11" s="159"/>
-      <c r="J11" s="159"/>
-      <c r="K11" s="159"/>
-      <c r="M11" s="100" t="s">
+      <c r="H11" s="157"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="157"/>
+      <c r="K11" s="157"/>
+      <c r="M11" s="98" t="s">
         <v>170</v>
       </c>
-      <c r="N11" s="101"/>
+      <c r="N11" s="99"/>
     </row>
     <row r="12" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A12" s="96"/>
-      <c r="B12" s="97"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="97"/>
-      <c r="G12" s="98" t="s">
+      <c r="A12" s="94"/>
+      <c r="B12" s="95"/>
+      <c r="D12" s="94"/>
+      <c r="E12" s="95"/>
+      <c r="G12" s="96" t="s">
         <v>156</v>
       </c>
-      <c r="H12" s="98" t="s">
+      <c r="H12" s="96" t="s">
         <v>157</v>
       </c>
-      <c r="I12" s="98" t="s">
+      <c r="I12" s="96" t="s">
         <v>105</v>
       </c>
-      <c r="J12" s="99" t="s">
+      <c r="J12" s="97" t="s">
         <v>158</v>
       </c>
-      <c r="K12" s="99" t="s">
+      <c r="K12" s="97" t="s">
         <v>159</v>
       </c>
-      <c r="M12" s="100" t="s">
+      <c r="M12" s="98" t="s">
         <v>171</v>
       </c>
-      <c r="N12" s="101"/>
+      <c r="N12" s="99"/>
     </row>
     <row r="13" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="D13" s="96"/>
-      <c r="E13" s="97"/>
-      <c r="G13" s="98" t="s">
+      <c r="A13" s="94"/>
+      <c r="B13" s="95"/>
+      <c r="D13" s="94"/>
+      <c r="E13" s="95"/>
+      <c r="G13" s="96" t="s">
         <v>172</v>
       </c>
-      <c r="H13" s="96">
+      <c r="H13" s="94">
         <v>1</v>
       </c>
-      <c r="I13" s="96"/>
-      <c r="J13" s="96"/>
-      <c r="K13" s="99">
+      <c r="I13" s="94"/>
+      <c r="J13" s="94"/>
+      <c r="K13" s="97">
         <f>(H13*3)+(I13*4)+(J13*6)</f>
         <v>3</v>
       </c>
-      <c r="M13" s="100" t="s">
+      <c r="M13" s="98" t="s">
         <v>173</v>
       </c>
-      <c r="N13" s="101"/>
+      <c r="N13" s="99"/>
       <c r="W13" s="4" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A14" s="96"/>
-      <c r="B14" s="97"/>
-      <c r="D14" s="96"/>
-      <c r="E14" s="97"/>
-      <c r="G14" s="98" t="s">
+      <c r="A14" s="94"/>
+      <c r="B14" s="95"/>
+      <c r="D14" s="94"/>
+      <c r="E14" s="95"/>
+      <c r="G14" s="96" t="s">
         <v>175</v>
       </c>
-      <c r="H14" s="96"/>
-      <c r="I14" s="96"/>
-      <c r="J14" s="96"/>
-      <c r="K14" s="99">
+      <c r="H14" s="94"/>
+      <c r="I14" s="94"/>
+      <c r="J14" s="94"/>
+      <c r="K14" s="97">
         <f>(H14*4)+(I14*5)+(J14*7)</f>
         <v>0</v>
       </c>
-      <c r="M14" s="100" t="s">
+      <c r="M14" s="98" t="s">
         <v>176</v>
       </c>
-      <c r="N14" s="101"/>
+      <c r="N14" s="99"/>
     </row>
     <row r="15" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A15" s="96"/>
-      <c r="B15" s="97"/>
-      <c r="D15" s="96"/>
-      <c r="E15" s="97"/>
-      <c r="G15" s="98" t="s">
+      <c r="A15" s="94"/>
+      <c r="B15" s="95"/>
+      <c r="D15" s="94"/>
+      <c r="E15" s="95"/>
+      <c r="G15" s="96" t="s">
         <v>177</v>
       </c>
-      <c r="H15" s="96">
+      <c r="H15" s="94">
         <v>1</v>
       </c>
-      <c r="I15" s="96"/>
-      <c r="J15" s="96"/>
-      <c r="K15" s="99">
+      <c r="I15" s="94"/>
+      <c r="J15" s="94"/>
+      <c r="K15" s="97">
         <f>(H15*3)+(I15*4)+(J15*6)</f>
         <v>3</v>
       </c>
-      <c r="M15" s="100" t="s">
+      <c r="M15" s="98" t="s">
         <v>178</v>
       </c>
-      <c r="N15" s="101"/>
+      <c r="N15" s="99"/>
     </row>
     <row r="16" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="96"/>
-      <c r="B16" s="97"/>
-      <c r="D16" s="96"/>
-      <c r="E16" s="97"/>
-      <c r="G16" s="160" t="s">
+      <c r="A16" s="94"/>
+      <c r="B16" s="95"/>
+      <c r="D16" s="94"/>
+      <c r="E16" s="95"/>
+      <c r="G16" s="158" t="s">
         <v>179</v>
       </c>
-      <c r="H16" s="160"/>
-      <c r="I16" s="160"/>
-      <c r="J16" s="160"/>
-      <c r="K16" s="102">
+      <c r="H16" s="158"/>
+      <c r="I16" s="158"/>
+      <c r="J16" s="158"/>
+      <c r="K16" s="100">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
       </c>
-      <c r="M16" s="100" t="s">
+      <c r="M16" s="98" t="s">
         <v>180</v>
       </c>
-      <c r="N16" s="101"/>
+      <c r="N16" s="99"/>
     </row>
     <row r="17" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A17" s="96"/>
-      <c r="B17" s="97"/>
-      <c r="D17" s="96"/>
-      <c r="E17" s="97"/>
-      <c r="M17" s="100" t="s">
+      <c r="A17" s="94"/>
+      <c r="B17" s="95"/>
+      <c r="D17" s="94"/>
+      <c r="E17" s="95"/>
+      <c r="M17" s="98" t="s">
         <v>181</v>
       </c>
-      <c r="N17" s="101"/>
+      <c r="N17" s="99"/>
     </row>
     <row r="18" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A18" s="96"/>
-      <c r="B18" s="97"/>
-      <c r="D18" s="96"/>
-      <c r="E18" s="97"/>
-      <c r="M18" s="100" t="s">
+      <c r="A18" s="94"/>
+      <c r="B18" s="95"/>
+      <c r="D18" s="94"/>
+      <c r="E18" s="95"/>
+      <c r="M18" s="98" t="s">
         <v>182</v>
       </c>
-      <c r="N18" s="101"/>
+      <c r="N18" s="99"/>
     </row>
     <row r="19" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A19" s="96"/>
-      <c r="B19" s="97"/>
-      <c r="D19" s="96"/>
-      <c r="E19" s="97"/>
-      <c r="M19" s="100" t="s">
+      <c r="A19" s="94"/>
+      <c r="B19" s="95"/>
+      <c r="D19" s="94"/>
+      <c r="E19" s="95"/>
+      <c r="M19" s="98" t="s">
         <v>183</v>
       </c>
-      <c r="N19" s="101"/>
+      <c r="N19" s="99"/>
     </row>
     <row r="20" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A20" s="96"/>
-      <c r="B20" s="97"/>
-      <c r="D20" s="96"/>
-      <c r="E20" s="97"/>
-      <c r="M20" s="100" t="s">
+      <c r="A20" s="94"/>
+      <c r="B20" s="95"/>
+      <c r="D20" s="94"/>
+      <c r="E20" s="95"/>
+      <c r="M20" s="98" t="s">
         <v>184</v>
       </c>
-      <c r="N20" s="101"/>
+      <c r="N20" s="99"/>
     </row>
     <row r="21" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="M21" s="100" t="s">
+      <c r="M21" s="98" t="s">
         <v>185</v>
       </c>
-      <c r="N21" s="101"/>
+      <c r="N21" s="99"/>
     </row>
     <row r="22" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="M22" s="100" t="s">
+      <c r="M22" s="98" t="s">
         <v>186</v>
       </c>
-      <c r="N22" s="101"/>
+      <c r="N22" s="99"/>
     </row>
     <row r="23" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="M23" s="103" t="s">
+      <c r="M23" s="101" t="s">
         <v>187</v>
       </c>
-      <c r="N23" s="104">
+      <c r="N23" s="102">
         <f>SUM(N9:N22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="M24" s="103" t="s">
+      <c r="M24" s="101" t="s">
         <v>188</v>
       </c>
-      <c r="N24" s="102">
+      <c r="N24" s="100">
         <f>(N23*0.01)+0.65</f>
         <v>0.65</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="M25" s="103" t="s">
+      <c r="M25" s="101" t="s">
         <v>189</v>
       </c>
-      <c r="N25" s="105">
+      <c r="N25" s="103">
         <f>K16*N24</f>
         <v>9.1</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="M26" s="103" t="s">
+      <c r="M26" s="101" t="s">
         <v>190</v>
       </c>
-      <c r="N26" s="106">
+      <c r="N26" s="104">
         <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.25">
-      <c r="M27" s="107" t="s">
+      <c r="M27" s="105" t="s">
         <v>191</v>
       </c>
-      <c r="N27" s="108">
+      <c r="N27" s="106">
         <f>N25*N26</f>
         <v>172.9</v>
       </c>
@@ -11339,74 +11419,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="161" t="s">
+      <c r="A1" s="159" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="161"/>
-      <c r="E1" s="161"/>
-      <c r="F1" s="161"/>
-      <c r="G1" s="161"/>
-      <c r="H1" s="161"/>
-      <c r="I1" s="161"/>
-      <c r="J1" s="161"/>
-      <c r="K1" s="161"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="161"/>
+      <c r="B1" s="159"/>
+      <c r="C1" s="159"/>
+      <c r="D1" s="159"/>
+      <c r="E1" s="159"/>
+      <c r="F1" s="159"/>
+      <c r="G1" s="159"/>
+      <c r="H1" s="159"/>
+      <c r="I1" s="159"/>
+      <c r="J1" s="159"/>
+      <c r="K1" s="159"/>
+      <c r="L1" s="159"/>
+      <c r="M1" s="159"/>
+      <c r="N1" s="159"/>
     </row>
     <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="167" t="s">
+      <c r="A3" s="165" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="167"/>
-      <c r="C3" s="167"/>
-      <c r="E3" s="167" t="s">
+      <c r="B3" s="165"/>
+      <c r="C3" s="165"/>
+      <c r="E3" s="165" t="s">
         <v>192</v>
       </c>
-      <c r="F3" s="167"/>
-      <c r="G3" s="167"/>
-      <c r="H3" s="167"/>
-      <c r="I3" s="167"/>
-      <c r="J3" s="167"/>
-      <c r="K3" s="167"/>
-      <c r="L3" s="167"/>
-      <c r="M3" s="167"/>
-      <c r="N3" s="167"/>
+      <c r="F3" s="165"/>
+      <c r="G3" s="165"/>
+      <c r="H3" s="165"/>
+      <c r="I3" s="165"/>
+      <c r="J3" s="165"/>
+      <c r="K3" s="165"/>
+      <c r="L3" s="165"/>
+      <c r="M3" s="165"/>
+      <c r="N3" s="165"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="107" t="s">
         <v>193</v>
       </c>
-      <c r="B4" s="110">
+      <c r="B4" s="108">
         <f>'#Estimativa-APF#'!$N$27</f>
         <v>172.9</v>
       </c>
       <c r="C4" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="168" t="s">
+      <c r="E4" s="166" t="s">
         <v>194</v>
       </c>
-      <c r="F4" s="166" t="s">
+      <c r="F4" s="164" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="166"/>
-      <c r="H4" s="166" t="s">
+      <c r="G4" s="164"/>
+      <c r="H4" s="164" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="166"/>
-      <c r="J4" s="166" t="s">
+      <c r="I4" s="164"/>
+      <c r="J4" s="164" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="166"/>
-      <c r="L4" s="166" t="s">
+      <c r="K4" s="164"/>
+      <c r="L4" s="164" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="166"/>
-      <c r="N4" s="111"/>
+      <c r="M4" s="164"/>
+      <c r="N4" s="109"/>
     </row>
     <row r="5" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
@@ -11418,68 +11498,68 @@
       <c r="C5" s="38" t="s">
         <v>195</v>
       </c>
-      <c r="E5" s="168"/>
-      <c r="F5" s="166" t="s">
+      <c r="E5" s="166"/>
+      <c r="F5" s="164" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="166"/>
-      <c r="H5" s="166" t="s">
+      <c r="G5" s="164"/>
+      <c r="H5" s="164" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="166"/>
-      <c r="J5" s="166" t="s">
+      <c r="I5" s="164"/>
+      <c r="J5" s="164" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="166"/>
-      <c r="L5" s="166" t="s">
+      <c r="K5" s="164"/>
+      <c r="L5" s="164" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="166"/>
+      <c r="M5" s="164"/>
       <c r="N5" s="41" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="112" t="s">
+      <c r="A6" s="110" t="s">
         <v>197</v>
       </c>
-      <c r="B6" s="113">
+      <c r="B6" s="111">
         <f>B4+(B4*B5)</f>
         <v>172.9</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="168"/>
-      <c r="F6" s="114">
+      <c r="E6" s="166"/>
+      <c r="F6" s="112">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
       </c>
-      <c r="G6" s="115">
+      <c r="G6" s="113">
         <v>0.05</v>
       </c>
-      <c r="H6" s="114">
+      <c r="H6" s="112">
         <f>B4*I6</f>
         <v>34.580000000000005</v>
       </c>
-      <c r="I6" s="115">
+      <c r="I6" s="113">
         <v>0.2</v>
       </c>
-      <c r="J6" s="114">
+      <c r="J6" s="112">
         <f>B4*K6</f>
         <v>112.38500000000001</v>
       </c>
-      <c r="K6" s="115">
+      <c r="K6" s="113">
         <v>0.65</v>
       </c>
-      <c r="L6" s="114">
+      <c r="L6" s="112">
         <f>B4*M6</f>
         <v>17.290000000000003</v>
       </c>
-      <c r="M6" s="115">
+      <c r="M6" s="113">
         <v>0.1</v>
       </c>
-      <c r="N6" s="114"/>
+      <c r="N6" s="112"/>
     </row>
     <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="30" t="s">
@@ -11489,38 +11569,38 @@
         <v>1</v>
       </c>
       <c r="C7" s="30"/>
-      <c r="E7" s="116" t="s">
+      <c r="E7" s="114" t="s">
         <v>199</v>
       </c>
-      <c r="F7" s="114">
+      <c r="F7" s="112">
         <f>F6*G7</f>
         <v>4.7547500000000014</v>
       </c>
-      <c r="G7" s="115">
+      <c r="G7" s="113">
         <v>0.55000000000000004</v>
       </c>
-      <c r="H7" s="114">
+      <c r="H7" s="112">
         <f>H6*I7</f>
         <v>10.374000000000001</v>
       </c>
-      <c r="I7" s="115">
+      <c r="I7" s="113">
         <v>0.3</v>
       </c>
-      <c r="J7" s="114">
+      <c r="J7" s="112">
         <f>J6*K7</f>
         <v>13.4862</v>
       </c>
-      <c r="K7" s="115">
+      <c r="K7" s="113">
         <v>0.12</v>
       </c>
-      <c r="L7" s="114">
+      <c r="L7" s="112">
         <f>L6*M7</f>
         <v>0.86450000000000016</v>
       </c>
-      <c r="M7" s="115">
+      <c r="M7" s="113">
         <v>0.05</v>
       </c>
-      <c r="N7" s="117">
+      <c r="N7" s="115">
         <f>SUM(F7,H7,J7,L7)</f>
         <v>29.47945</v>
       </c>
@@ -11535,38 +11615,38 @@
       <c r="C8" s="30" t="s">
         <v>201</v>
       </c>
-      <c r="E8" s="116" t="s">
+      <c r="E8" s="114" t="s">
         <v>202</v>
       </c>
-      <c r="F8" s="114">
+      <c r="F8" s="112">
         <f>F6*G8</f>
         <v>1.2967500000000001</v>
       </c>
-      <c r="G8" s="115">
+      <c r="G8" s="113">
         <v>0.15</v>
       </c>
-      <c r="H8" s="114">
+      <c r="H8" s="112">
         <f>H6*I8</f>
         <v>6.9160000000000013</v>
       </c>
-      <c r="I8" s="115">
+      <c r="I8" s="113">
         <v>0.2</v>
       </c>
-      <c r="J8" s="114">
+      <c r="J8" s="112">
         <f>J6*K8</f>
         <v>11.238500000000002</v>
       </c>
-      <c r="K8" s="115">
+      <c r="K8" s="113">
         <v>0.1</v>
       </c>
-      <c r="L8" s="114">
+      <c r="L8" s="112">
         <f>L6*M8</f>
         <v>0.86450000000000016</v>
       </c>
-      <c r="M8" s="115">
+      <c r="M8" s="113">
         <v>0.05</v>
       </c>
-      <c r="N8" s="117">
+      <c r="N8" s="115">
         <f>SUM(F8,H8,J8,L8)</f>
         <v>20.315750000000001</v>
       </c>
@@ -11581,348 +11661,348 @@
       <c r="C9" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="116" t="s">
+      <c r="E9" s="114" t="s">
         <v>204</v>
       </c>
-      <c r="F9" s="114">
+      <c r="F9" s="112">
         <f>F6*G9</f>
         <v>0.17290000000000003</v>
       </c>
-      <c r="G9" s="115">
+      <c r="G9" s="113">
         <v>0.02</v>
       </c>
-      <c r="H9" s="114">
+      <c r="H9" s="112">
         <f>H6*I9</f>
         <v>6.9160000000000013</v>
       </c>
-      <c r="I9" s="115">
+      <c r="I9" s="113">
         <v>0.2</v>
       </c>
-      <c r="J9" s="114">
+      <c r="J9" s="112">
         <f>J6*K9</f>
         <v>44.954000000000008</v>
       </c>
-      <c r="K9" s="115">
+      <c r="K9" s="113">
         <v>0.4</v>
       </c>
-      <c r="L9" s="114">
+      <c r="L9" s="112">
         <f>L6*M9</f>
         <v>2.5935000000000001</v>
       </c>
-      <c r="M9" s="115">
+      <c r="M9" s="113">
         <v>0.15</v>
       </c>
-      <c r="N9" s="117">
+      <c r="N9" s="115">
         <f>SUM(F9,H9,J9,L9)</f>
         <v>54.636400000000009</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="118" t="s">
+      <c r="A10" s="116" t="s">
         <v>205</v>
       </c>
-      <c r="B10" s="119">
+      <c r="B10" s="117">
         <f>(B7*B8)*B9</f>
         <v>80</v>
       </c>
-      <c r="C10" s="118" t="s">
+      <c r="C10" s="116" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="116" t="s">
+      <c r="E10" s="114" t="s">
         <v>206</v>
       </c>
-      <c r="F10" s="114">
+      <c r="F10" s="112">
         <f>F6*G10</f>
         <v>0.43225000000000008</v>
       </c>
-      <c r="G10" s="115">
+      <c r="G10" s="113">
         <v>0.05</v>
       </c>
-      <c r="H10" s="114">
+      <c r="H10" s="112">
         <f>H6*I10</f>
         <v>2.7664000000000004</v>
       </c>
-      <c r="I10" s="115">
+      <c r="I10" s="113">
         <v>0.08</v>
       </c>
-      <c r="J10" s="114">
+      <c r="J10" s="112">
         <f>J6*K10</f>
         <v>11.238500000000002</v>
       </c>
-      <c r="K10" s="115">
+      <c r="K10" s="113">
         <v>0.1</v>
       </c>
-      <c r="L10" s="114">
+      <c r="L10" s="112">
         <f>L6*M10</f>
         <v>1.7290000000000003</v>
       </c>
-      <c r="M10" s="115">
+      <c r="M10" s="113">
         <v>0.1</v>
       </c>
-      <c r="N10" s="117">
+      <c r="N10" s="115">
         <f>SUM(F10,H10,J10,L10)</f>
         <v>16.166150000000002</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="109" t="s">
+      <c r="A11" s="107" t="s">
         <v>207</v>
       </c>
-      <c r="B11" s="120">
+      <c r="B11" s="118">
         <f>B6/B10*2</f>
         <v>4.3224999999999998</v>
       </c>
-      <c r="C11" s="109" t="s">
+      <c r="C11" s="107" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="116" t="s">
+      <c r="E11" s="114" t="s">
         <v>208</v>
       </c>
-      <c r="F11" s="114">
+      <c r="F11" s="112">
         <f>F6*G11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="115">
+      <c r="G11" s="113">
         <v>0</v>
       </c>
-      <c r="H11" s="114">
+      <c r="H11" s="112">
         <f>H6*I11</f>
         <v>0.6916000000000001</v>
       </c>
-      <c r="I11" s="115">
+      <c r="I11" s="113">
         <v>0.02</v>
       </c>
-      <c r="J11" s="114">
+      <c r="J11" s="112">
         <f>J6*K11</f>
         <v>5.619250000000001</v>
       </c>
-      <c r="K11" s="115">
+      <c r="K11" s="113">
         <v>0.05</v>
       </c>
-      <c r="L11" s="114">
+      <c r="L11" s="112">
         <f>L6*M11</f>
         <v>1.7290000000000003</v>
       </c>
-      <c r="M11" s="115">
+      <c r="M11" s="113">
         <v>0.1</v>
       </c>
-      <c r="N11" s="117">
+      <c r="N11" s="115">
         <f>SUM(F11,H11,J11,L11)</f>
         <v>8.0398500000000013</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="109" t="s">
+      <c r="A12" s="107" t="s">
         <v>209</v>
       </c>
-      <c r="B12" s="120">
+      <c r="B12" s="118">
         <f>B11/4</f>
         <v>1.0806249999999999</v>
       </c>
-      <c r="C12" s="109" t="s">
+      <c r="C12" s="107" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="121" t="s">
+      <c r="E12" s="119" t="s">
         <v>210</v>
       </c>
-      <c r="F12" s="122">
+      <c r="F12" s="120">
         <f t="shared" ref="F12:M12" si="0">SUM(F7:F11)</f>
         <v>6.6566500000000017</v>
       </c>
-      <c r="G12" s="123">
+      <c r="G12" s="121">
         <f t="shared" si="0"/>
         <v>0.77000000000000013</v>
       </c>
-      <c r="H12" s="122">
+      <c r="H12" s="120">
         <f t="shared" si="0"/>
         <v>27.664000000000005</v>
       </c>
-      <c r="I12" s="123">
+      <c r="I12" s="121">
         <f t="shared" si="0"/>
         <v>0.79999999999999993</v>
       </c>
-      <c r="J12" s="122">
+      <c r="J12" s="120">
         <f t="shared" si="0"/>
         <v>86.536450000000002</v>
       </c>
-      <c r="K12" s="123">
+      <c r="K12" s="121">
         <f t="shared" si="0"/>
         <v>0.77</v>
       </c>
-      <c r="L12" s="122">
+      <c r="L12" s="120">
         <f t="shared" si="0"/>
         <v>7.7805000000000009</v>
       </c>
-      <c r="M12" s="123">
+      <c r="M12" s="121">
         <f t="shared" si="0"/>
         <v>0.44999999999999996</v>
       </c>
-      <c r="N12" s="121"/>
+      <c r="N12" s="119"/>
     </row>
     <row r="13" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="118" t="s">
+      <c r="A13" s="116" t="s">
         <v>211</v>
       </c>
-      <c r="B13" s="124">
+      <c r="B13" s="122">
         <f>B11/B9</f>
         <v>2.1612499999999999</v>
       </c>
-      <c r="C13" s="118" t="s">
+      <c r="C13" s="116" t="s">
         <v>212</v>
       </c>
-      <c r="E13" s="116" t="s">
+      <c r="E13" s="114" t="s">
         <v>213</v>
       </c>
-      <c r="F13" s="114">
+      <c r="F13" s="112">
         <f>F6*G13</f>
         <v>0.25935000000000002</v>
       </c>
-      <c r="G13" s="115">
+      <c r="G13" s="113">
         <v>0.03</v>
       </c>
-      <c r="H13" s="114">
+      <c r="H13" s="112">
         <f>H6*I13</f>
         <v>2.7664000000000004</v>
       </c>
-      <c r="I13" s="115">
+      <c r="I13" s="113">
         <v>0.08</v>
       </c>
-      <c r="J13" s="114">
+      <c r="J13" s="112">
         <f>J6*K13</f>
         <v>14.610050000000001</v>
       </c>
-      <c r="K13" s="115">
+      <c r="K13" s="113">
         <v>0.13</v>
       </c>
-      <c r="L13" s="114">
+      <c r="L13" s="112">
         <f>L6*M13</f>
         <v>5.1870000000000003</v>
       </c>
-      <c r="M13" s="115">
+      <c r="M13" s="113">
         <v>0.3</v>
       </c>
-      <c r="N13" s="117">
+      <c r="N13" s="115">
         <f>SUM(F13,H13,J13,L13)</f>
         <v>22.822800000000004</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E14" s="116" t="s">
+      <c r="E14" s="114" t="s">
         <v>214</v>
       </c>
-      <c r="F14" s="114">
+      <c r="F14" s="112">
         <f>F6*G14</f>
         <v>1.7290000000000003</v>
       </c>
-      <c r="G14" s="115">
+      <c r="G14" s="113">
         <v>0.2</v>
       </c>
-      <c r="H14" s="114">
+      <c r="H14" s="112">
         <f>H6*I14</f>
         <v>4.1496000000000004</v>
       </c>
-      <c r="I14" s="115">
+      <c r="I14" s="113">
         <v>0.12</v>
       </c>
-      <c r="J14" s="114">
+      <c r="J14" s="112">
         <f>J6*K14</f>
         <v>11.238500000000002</v>
       </c>
-      <c r="K14" s="115">
+      <c r="K14" s="113">
         <v>0.1</v>
       </c>
-      <c r="L14" s="114">
+      <c r="L14" s="112">
         <f>L6*M14</f>
         <v>4.3225000000000007</v>
       </c>
-      <c r="M14" s="115">
+      <c r="M14" s="113">
         <v>0.25</v>
       </c>
-      <c r="N14" s="117">
+      <c r="N14" s="115">
         <f>SUM(F14,H14,J14,L14)</f>
         <v>21.439600000000002</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="E15" s="121" t="s">
+      <c r="E15" s="119" t="s">
         <v>215</v>
       </c>
-      <c r="F15" s="122">
+      <c r="F15" s="120">
         <f t="shared" ref="F15:M15" si="1">SUM(F13:F14)</f>
         <v>1.9883500000000003</v>
       </c>
-      <c r="G15" s="123">
+      <c r="G15" s="121">
         <f t="shared" si="1"/>
         <v>0.23</v>
       </c>
-      <c r="H15" s="122">
+      <c r="H15" s="120">
         <f t="shared" si="1"/>
         <v>6.9160000000000004</v>
       </c>
-      <c r="I15" s="123">
+      <c r="I15" s="121">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="J15" s="122">
+      <c r="J15" s="120">
         <f t="shared" si="1"/>
         <v>25.848550000000003</v>
       </c>
-      <c r="K15" s="123">
+      <c r="K15" s="121">
         <f t="shared" si="1"/>
         <v>0.23</v>
       </c>
-      <c r="L15" s="122">
+      <c r="L15" s="120">
         <f t="shared" si="1"/>
         <v>9.509500000000001</v>
       </c>
-      <c r="M15" s="123">
+      <c r="M15" s="121">
         <f t="shared" si="1"/>
         <v>0.55000000000000004</v>
       </c>
-      <c r="N15" s="121"/>
+      <c r="N15" s="119"/>
     </row>
     <row r="16" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="167" t="s">
+      <c r="A16" s="165" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="167"/>
-      <c r="C16" s="167"/>
+      <c r="B16" s="165"/>
+      <c r="C16" s="165"/>
       <c r="E16" s="41" t="s">
         <v>216</v>
       </c>
-      <c r="F16" s="125">
+      <c r="F16" s="123">
         <f t="shared" ref="F16:M16" si="2">F12+F15</f>
         <v>8.6450000000000014</v>
       </c>
-      <c r="G16" s="126">
+      <c r="G16" s="124">
         <f t="shared" si="2"/>
         <v>1.0000000000000002</v>
       </c>
-      <c r="H16" s="125">
+      <c r="H16" s="123">
         <f t="shared" si="2"/>
         <v>34.580000000000005</v>
       </c>
-      <c r="I16" s="126">
+      <c r="I16" s="124">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="J16" s="125">
+      <c r="J16" s="123">
         <f t="shared" si="2"/>
         <v>112.38500000000001</v>
       </c>
-      <c r="K16" s="126">
+      <c r="K16" s="124">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="L16" s="125">
+      <c r="L16" s="123">
         <f t="shared" si="2"/>
         <v>17.290000000000003</v>
       </c>
-      <c r="M16" s="126">
+      <c r="M16" s="124">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="N16" s="127">
+      <c r="N16" s="125">
         <f>SUM(N7:N11,N13,N14)</f>
         <v>172.90000000000003</v>
       </c>
@@ -11931,11 +12011,11 @@
       <c r="A17" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="B17" s="128">
+      <c r="B17" s="126">
         <v>20</v>
       </c>
       <c r="C17" s="38"/>
-      <c r="N17" s="72"/>
+      <c r="N17" s="70"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="30" t="s">
@@ -11946,8 +12026,8 @@
         <v>3458</v>
       </c>
       <c r="C18" s="38"/>
-      <c r="L18" s="72"/>
-      <c r="N18" s="72"/>
+      <c r="L18" s="70"/>
+      <c r="N18" s="70"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="s">
@@ -11957,7 +12037,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="38"/>
-      <c r="N19" s="72"/>
+      <c r="N19" s="70"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="30" t="s">
@@ -11968,19 +12048,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="38"/>
-      <c r="L20" s="72"/>
-      <c r="N20" s="72"/>
+      <c r="L20" s="70"/>
+      <c r="N20" s="70"/>
     </row>
     <row r="21" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="B21" s="129">
+      <c r="B21" s="127">
         <f>B18+B20</f>
         <v>3458</v>
       </c>
       <c r="C21" s="38"/>
-      <c r="N21" s="72"/>
+      <c r="N21" s="70"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="s">
@@ -11990,7 +12070,7 @@
         <v>0.2</v>
       </c>
       <c r="C22" s="38"/>
-      <c r="J22" s="72"/>
+      <c r="J22" s="70"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="s">
@@ -12006,23 +12086,23 @@
       <c r="A24" s="26" t="s">
         <v>218</v>
       </c>
-      <c r="B24" s="129">
+      <c r="B24" s="127">
         <f>B21+B23</f>
         <v>4149.6000000000004</v>
       </c>
       <c r="C24" s="38"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J26" s="72"/>
+      <c r="J26" s="70"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J27" s="72"/>
+      <c r="J27" s="70"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N28" s="72"/>
+      <c r="N28" s="70"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N29" s="72"/>
+      <c r="N29" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>